<commit_message>
Sync the Evidence Map from its Google Sheet automatically
An hourly GitHub Action (also runnable on demand) downloads the Sheet's
published studies and topics CSVs, validates them, writes _data/, and
commits any changes, then requests a Pages build.

- scripts/sync_evidence_map.py rejects a tab that returns a web page,
  has a changed header, or has duplicate ids, leaving the current data
  untouched; skips rows without an id; ignores extra columns; strips
  BOM/CRLF; warns about topic ids missing from the topics tab
- Draft studies now stay off the public site until marked published,
  since Sheet edits go live without a manual step
- docs/EVIDENCE-MAP.md covers publishing the tabs, setting the two
  URLs, and troubleshooting; the backup workbook's Instructions tab and
  the extraction prompt match the new flow

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LjTRSkq14Nqt674Y3357uL
</commit_message>
<xml_diff>
--- a/docs/curation/evidence-map-curation.xlsx
+++ b/docs/curation/evidence-map-curation.xlsx
@@ -471,128 +471,128 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>TO PUBLISH</t>
+          <t>HOW IT REACHES THE SITE</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>1. Select the 'studies' tab, then File &gt; Download &gt; Comma-separated values (.csv).</t>
+          <t>The 'studies' and 'topics' tabs are published to the web as CSV. A GitHub Action copies them to the site every hour.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2. Do the same for the 'topics' tab.</t>
+          <t>Changes appear within about an hour. To update sooner: GitHub repo &gt; Actions &gt; Sync Evidence Map &gt; Run workflow.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>3. Rename the downloads to studies.csv and topics.csv.</t>
+          <t>Published tabs can be read by anyone with the links, so keep private notes out of them.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>4. In the GitHub repo, open the _data folder, choose Add file &gt; Upload files, upload both, and commit. The site updates in a minute or two.</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>TOPICS TAB (one row per topic)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>TOPICS TAB (one row per topic)</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>id: short lowercase id with hyphens, e.g. fmt, ibs, dietary-fiber. Never change an id once studies use it.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>id: short lowercase id with hyphens, e.g. fmt, ibs, dietary-fiber. Never change an id once studies use it.</t>
+          <t>name: display name.  type: treatment, condition, or mechanism.  summary: one sentence.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>name: display name.  type: treatment, condition, or mechanism.  summary: one sentence.</t>
+          <t>entry: optional Knowledge Base file name without .md (e.g. fecal-microbiota-transplantation) to link the topic to that entry.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>entry: optional Knowledge Base file name without .md (e.g. fecal-microbiota-transplantation) to link the topic to that entry.</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>STUDIES TAB (one row per article)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>STUDIES TAB (one row per article)</t>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>id: unique id, e.g. vannood-2013.  treatments / conditions / other_topics: topic ids separated by semicolons, e.g. fmt;probiotics</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>id: unique id, e.g. vannood-2013.  treatments / conditions / other_topics: topic ids separated by semicolons, e.g. fmt;probiotics</t>
+          <t>other_topics is for mechanisms (and anything else that is not a treatment or condition).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>other_topics is for mechanisms (and anything else that is not a treatment or condition).</t>
+          <t>finding: benefit, no-effect, mixed, harm, or n/a.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>finding: benefit, no-effect, mixed, harm, or n/a.</t>
+          <t>conclusion: the study's main conclusion in 1-2 sentences.  relevance: why it matters to the broader topic.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>conclusion: the study's main conclusion in 1-2 sentences.  relevance: why it matters to the broader topic.</t>
+          <t>status: published (shown on the site), draft (not shown until published), hidden (not shown), or example (sample rows; delete them once real rows exist).</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>status: published, draft (shows a Draft badge), hidden (left off the site), or example (sample rows; delete them once real rows exist).</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Every topic id used on the studies tab must exist on the topics tab. If one is missing, the Evidence Map shows a data-check warning naming it.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Every topic id used on the studies tab must exist on the topics tab. If one is missing, the Evidence Map shows a data-check warning naming it.</t>
+          <t>Every row needs a unique id; rows without one are skipped, and duplicate ids stop the sync until fixed.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Keep the header row exactly as is: the website reads columns by these names.</t>
+          <t>Keep the header row exactly as is: the sync rejects a tab whose column names change.</t>
         </is>
       </c>
     </row>

</xml_diff>